<commit_message>
Apply trailer local main ship (CRM notifications, order adjustments, finance/HRMS/maintenance).
Port unpushed trailer commits c8599f0d + c846177e onto feature/trailer-erp-2-form.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/implementation/client-csv-import/FOS_ERP_Client_Data_Collection.xlsx
+++ b/docs/implementation/client-csv-import/FOS_ERP_Client_Data_Collection.xlsx
@@ -85,7 +85,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-07-29</t>
+    <t>2026-08-03</t>
   </si>
   <si>
     <t>Section</t>
@@ -463,7 +463,7 @@
     <t>08_chart_of_accounts.csv</t>
   </si>
   <si>
-    <t>Collection sheet — matches CoA UI template. No production API CSV import yet. Account Type: Group|Posting. Category: Asset|Liability|Equity|Income|Expense.</t>
+    <t>Live API CSV import (Accounting → Chart of Accounts → Import). Scoped to legal entity. Account Type: Group|Posting. Category: Asset|Liability|Equity|Income|Expense. Parent by Account Code. Duplicate mode: skip|update|reject.</t>
   </si>
   <si>
     <t>09_Warehouses</t>
@@ -2800,7 +2800,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <tabColor rgb="FF6D4C41"/>
+    <tabColor rgb="FF00695C"/>
   </sheetPr>
   <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -4867,7 +4867,7 @@
         <v>144</v>
       </c>
       <c r="C10" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D10" t="s">
         <v>145</v>

</xml_diff>